<commit_message>
Imported and set up most of the new HUD.
</commit_message>
<xml_diff>
--- a/Production/Flipper Ticklist.xlsx
+++ b/Production/Flipper Ticklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\The-Flipper-Framework\Production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37027090-1D04-496B-BA31-29CCDC10D55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78087C9A-8D74-4F3D-A33C-658F634E9040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="660" windowWidth="19440" windowHeight="14880" xr2:uid="{85BE2389-3B13-409D-8678-A22E603B8D44}"/>
   </bookViews>
@@ -241,7 +241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment shrinkToFit="1"/>
@@ -285,9 +285,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1326,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -1367,12 +1364,12 @@
       <c r="F16" s="13">
         <v>5</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="13">
         <f>SUM(F16 - E16)</f>
         <v>3</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>